<commit_message>
updated several raw data files
</commit_message>
<xml_diff>
--- a/data/raw/GLNPO 2024 Spring/Huron/D100/HU 06 D100 Spring 2024 24GH00I13 Zoop.xlsx
+++ b/data/raw/GLNPO 2024 Spring/Huron/D100/HU 06 D100 Spring 2024 24GH00I13 Zoop.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmars\OneDrive\Desktop\CCM Work Files\GLNPO Zooplankton Database\data\raw\GLNPO 2024 Spring\Huron\D100\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{663B042D-75BF-4BA0-8828-55A5B1E758AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA6ECB93-2905-4031-9A08-FBDDF764A944}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1C48D42D-7BA5-4224-B0A1-A701E2F2CC95}"/>
   </bookViews>
@@ -20,7 +20,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="36" r:id="rId2"/>
+    <pivotCache cacheId="3" r:id="rId2"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -5720,7 +5720,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{98A5F4BA-EB0C-4D9A-915A-0AD56F614B0D}" name="PivotTable5" cacheId="36" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{98A5F4BA-EB0C-4D9A-915A-0AD56F614B0D}" name="PivotTable5" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="U2:Z17" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="18">
     <pivotField showAll="0"/>
@@ -6172,7 +6172,8 @@
   <cols>
     <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="25.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="30.44140625" customWidth="1"/>
+    <col min="12" max="12" width="12.77734375" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="27.6640625" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="17" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="6.88671875" bestFit="1" customWidth="1"/>
@@ -6236,7 +6237,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -6295,7 +6296,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -6638,7 +6639,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -6768,7 +6769,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -6898,7 +6899,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>18</v>
       </c>
@@ -7034,7 +7035,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -7549,7 +7550,7 @@
         <v>0.996</v>
       </c>
     </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>18</v>
       </c>
@@ -7786,7 +7787,7 @@
       </c>
       <c r="V25" s="8"/>
     </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>18</v>
       </c>
@@ -7948,7 +7949,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>18</v>
       </c>
@@ -8054,7 +8055,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>18</v>
       </c>
@@ -8266,7 +8267,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>18</v>
       </c>
@@ -8481,7 +8482,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>18</v>
       </c>
@@ -9276,7 +9277,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>18</v>
       </c>
@@ -9488,7 +9489,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>18</v>
       </c>
@@ -9594,7 +9595,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>18</v>
       </c>
@@ -9912,7 +9913,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>18</v>
       </c>
@@ -10230,7 +10231,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>18</v>
       </c>
@@ -10283,7 +10284,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>18</v>
       </c>
@@ -10601,7 +10602,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>18</v>
       </c>
@@ -10654,7 +10655,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>18</v>
       </c>
@@ -10919,7 +10920,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>18</v>
       </c>
@@ -10972,7 +10973,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>18</v>
       </c>
@@ -11237,7 +11238,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>18</v>
       </c>
@@ -11290,7 +11291,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>18</v>
       </c>
@@ -11661,7 +11662,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>18</v>
       </c>
@@ -11714,7 +11715,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>18</v>
       </c>
@@ -12138,7 +12139,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>18</v>
       </c>
@@ -12297,7 +12298,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>18</v>
       </c>
@@ -12509,7 +12510,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="115" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>18</v>
       </c>
@@ -12562,7 +12563,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>18</v>
       </c>
@@ -12986,7 +12987,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>18</v>
       </c>
@@ -13463,7 +13464,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="133" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>18</v>
       </c>
@@ -13516,7 +13517,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="134" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>18</v>
       </c>
@@ -14364,7 +14365,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="150" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>18</v>
       </c>
@@ -14417,7 +14418,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>18</v>
       </c>
@@ -14579,7 +14580,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>18</v>
       </c>
@@ -15003,7 +15004,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="162" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>18</v>
       </c>
@@ -15056,7 +15057,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="163" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>18</v>
       </c>
@@ -15215,7 +15216,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="166" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>18</v>
       </c>
@@ -15430,7 +15431,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>18</v>
       </c>
@@ -16490,7 +16491,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="190" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>18</v>
       </c>
@@ -16543,7 +16544,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="191" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>18</v>
       </c>
@@ -16861,7 +16862,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="197" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>18</v>
       </c>
@@ -17126,7 +17127,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="202" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>18</v>
       </c>
@@ -17179,7 +17180,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="203" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>18</v>
       </c>
@@ -17762,7 +17763,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="214" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>18</v>
       </c>
@@ -17815,7 +17816,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="215" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>18</v>
       </c>
@@ -18186,7 +18187,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="222" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>18</v>
       </c>
@@ -18239,7 +18240,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="223" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>18</v>
       </c>
@@ -18292,7 +18293,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="224" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>18</v>
       </c>
@@ -18345,7 +18346,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="225" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>18</v>
       </c>
@@ -18398,7 +18399,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="226" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>18</v>
       </c>
@@ -18504,7 +18505,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="228" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>18</v>
       </c>
@@ -18557,7 +18558,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="229" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>18</v>
       </c>
@@ -18663,7 +18664,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="231" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>18</v>
       </c>
@@ -18928,7 +18929,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="236" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>18</v>
       </c>
@@ -19087,7 +19088,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="239" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>18</v>
       </c>
@@ -19989,7 +19990,7 @@
       </c>
       <c r="R255" s="5"/>
     </row>
-    <row r="256" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A256" s="5" t="s">
         <v>18</v>
       </c>
@@ -20030,7 +20031,7 @@
         <v>63</v>
       </c>
       <c r="N256" s="5" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="O256" s="5" t="s">
         <v>38</v>
@@ -20043,7 +20044,7 @@
       </c>
       <c r="R256" s="5"/>
     </row>
-    <row r="257" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A257" s="5" t="s">
         <v>18</v>
       </c>
@@ -20084,7 +20085,7 @@
         <v>63</v>
       </c>
       <c r="N257" s="5" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="O257" s="5" t="s">
         <v>38</v>
@@ -20425,7 +20426,8 @@
   <autoFilter ref="A1:S263" xr:uid="{1701234F-357B-4975-B616-15E070902B9D}">
     <filterColumn colId="10">
       <filters>
-        <filter val="Diacyclops thomasi"/>
+        <filter val="Daphnia galeata mendotae"/>
+        <filter val="Daphnia spp."/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>